<commit_message>
fix: gate admin spells and clear staff perks on demote #644
- Add spell.role column and enforce in spell_cast
- Strip admin spells and super_hide when role drops to USER
- Clear saved super_hide on login for USER characters
</commit_message>
<xml_diff>
--- a/resources/table/spell.xlsx
+++ b/resources/table/spell.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="spell" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spell" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:F300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="6" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -494,7 +494,12 @@
           <t>message</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t># 구현</t>
         </is>
@@ -521,7 +526,12 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t># 구현</t>
         </is>
@@ -548,7 +558,12 @@
           <t>server</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t># 구현</t>
         </is>
@@ -575,7 +590,12 @@
           <t>갈 곳은? 동(1), 서(2), 남(3), 북(4)?</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -602,7 +622,12 @@
           <t>갈 곳은?(좌, 우)</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -629,7 +654,12 @@
           <t>출두할 대상은?</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -656,7 +686,12 @@
           <t>소환할 대상은?</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -678,7 +713,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -705,7 +745,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -727,7 +772,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -749,7 +799,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -776,7 +831,12 @@
           <t>할 말은?</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -803,7 +863,12 @@
           <t>할 말은?</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -830,7 +895,12 @@
           <t>할 말은?</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -857,7 +927,12 @@
           <t>할 말은?</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -879,56 +954,71 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>다리밟기</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>TARGET</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>TARGET</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">어디를? </t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>견우직녀축복</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>NORMAL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -955,7 +1045,12 @@
           <t>무기의 이름은?</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -982,7 +1077,12 @@
           <t>무기의 이름은?</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1009,7 +1109,12 @@
           <t>무기의 이름은?</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1036,7 +1141,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1058,7 +1168,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1080,7 +1195,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1102,7 +1222,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1124,7 +1249,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1146,7 +1276,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1168,7 +1303,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1190,7 +1330,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1212,7 +1357,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1234,7 +1384,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1256,7 +1411,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1278,7 +1438,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1300,7 +1465,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1322,7 +1492,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1344,7 +1519,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E36" s="1" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1366,7 +1546,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E37" s="1" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1388,7 +1573,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E38" s="1" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1410,7 +1600,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E39" s="1" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1432,7 +1627,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E40" s="1" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1454,7 +1654,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E41" s="1" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1476,7 +1681,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E42" s="1" t="inlineStr">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1503,7 +1713,12 @@
           <t>변신할 동물은?</t>
         </is>
       </c>
-      <c r="E43" s="1" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1530,7 +1745,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E44" s="1" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1557,7 +1777,12 @@
           <t>변신할 동물은?</t>
         </is>
       </c>
-      <c r="E45" s="1" t="inlineStr">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1584,7 +1809,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E46" s="1" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1611,7 +1841,12 @@
           <t>변신할 동물은?</t>
         </is>
       </c>
-      <c r="E47" s="1" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1638,7 +1873,12 @@
           <t>변신할 동물은?</t>
         </is>
       </c>
-      <c r="E48" s="1" t="inlineStr">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1660,7 +1900,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E49" s="1" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1687,7 +1932,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E50" s="1" t="inlineStr">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1709,7 +1959,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E51" s="1" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1731,6 +1986,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
@@ -1748,7 +2008,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E53" s="1" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1770,7 +2035,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E54" s="1" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1792,6 +2062,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
@@ -1809,7 +2084,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E56" s="1" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1831,7 +2111,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E57" s="1" t="inlineStr">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1853,7 +2138,12 @@
           <t>TARGET</t>
         </is>
       </c>
-      <c r="E58" s="1" t="inlineStr">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1875,7 +2165,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E59" s="1" t="inlineStr">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1897,7 +2192,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E60" s="1" t="inlineStr">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1919,7 +2219,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E61" s="1" t="inlineStr">
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1941,7 +2246,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E62" s="1" t="inlineStr">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1963,7 +2273,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E63" s="1" t="inlineStr">
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1985,7 +2300,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E64" s="1" t="inlineStr">
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2007,7 +2327,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E65" s="1" t="inlineStr">
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2029,6 +2354,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
@@ -2046,6 +2376,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
@@ -2063,7 +2398,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E68" s="1" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F68" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2090,7 +2430,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E69" s="1" t="inlineStr">
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F69" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2117,7 +2462,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E70" s="1" t="inlineStr">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2144,7 +2494,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E71" s="1" t="inlineStr">
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F71" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2171,7 +2526,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E72" s="1" t="inlineStr">
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F72" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2198,7 +2558,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E73" s="1" t="inlineStr">
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F73" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2225,7 +2590,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E74" s="1" t="inlineStr">
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F74" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2252,7 +2622,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E75" s="1" t="inlineStr">
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F75" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2279,7 +2654,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E76" s="1" t="inlineStr">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F76" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2306,7 +2686,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E77" s="1" t="inlineStr">
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F77" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2333,7 +2718,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E78" s="1" t="inlineStr">
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F78" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2360,7 +2750,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E79" s="1" t="inlineStr">
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F79" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2387,7 +2782,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E80" s="1" t="inlineStr">
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F80" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2414,7 +2814,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E81" s="1" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F81" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2441,7 +2846,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E82" s="1" t="inlineStr">
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F82" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2468,7 +2878,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E83" s="1" t="inlineStr">
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F83" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2495,7 +2910,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E84" s="1" t="inlineStr">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F84" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2522,7 +2942,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E85" s="1" t="inlineStr">
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F85" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2549,7 +2974,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E86" s="1" t="inlineStr">
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F86" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2576,7 +3006,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E87" s="1" t="inlineStr">
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F87" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2603,7 +3038,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E88" s="1" t="inlineStr">
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F88" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2630,7 +3070,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E89" s="1" t="inlineStr">
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F89" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2652,7 +3097,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E90" s="1" t="inlineStr">
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F90" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2674,7 +3124,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E91" s="1" t="inlineStr">
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F91" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2696,7 +3151,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E92" s="1" t="inlineStr">
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F92" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2718,7 +3178,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E93" s="1" t="inlineStr">
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F93" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2740,7 +3205,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E94" s="1" t="inlineStr">
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F94" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2762,7 +3232,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E95" s="1" t="inlineStr">
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F95" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2784,7 +3259,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E96" s="1" t="inlineStr">
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F96" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2806,7 +3286,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E97" s="1" t="inlineStr">
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F97" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2828,7 +3313,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E98" s="1" t="inlineStr">
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F98" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2850,7 +3340,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E99" s="1" t="inlineStr">
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F99" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2872,7 +3367,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E100" s="1" t="inlineStr">
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F100" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2894,7 +3394,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E101" s="1" t="inlineStr">
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F101" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2916,7 +3421,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E102" s="1" t="inlineStr">
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F102" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2938,7 +3448,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E103" s="1" t="inlineStr">
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F103" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2960,7 +3475,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E104" s="1" t="inlineStr">
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F104" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2982,7 +3502,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E105" s="1" t="inlineStr">
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F105" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3004,7 +3529,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E106" s="1" t="inlineStr">
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F106" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3026,7 +3556,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E107" s="1" t="inlineStr">
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F107" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3048,7 +3583,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E108" s="1" t="inlineStr">
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F108" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3070,7 +3610,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E109" s="1" t="inlineStr">
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F109" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3097,6 +3642,11 @@
           <t>대상은?</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
@@ -3119,7 +3669,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E111" s="1" t="inlineStr">
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F111" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3146,7 +3701,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E112" s="1" t="inlineStr">
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F112" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3168,7 +3728,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E113" s="1" t="inlineStr">
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F113" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3190,7 +3755,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E114" s="1" t="inlineStr">
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F114" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3217,7 +3787,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E115" s="1" t="inlineStr">
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F115" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3239,6 +3814,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
@@ -3261,6 +3841,11 @@
           <t>대상은?</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
@@ -3278,6 +3863,11 @@
           <t>TARGET</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
@@ -3300,7 +3890,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E119" s="1" t="inlineStr">
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F119" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3327,7 +3922,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E120" s="1" t="inlineStr">
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F120" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3354,7 +3954,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E121" s="1" t="inlineStr">
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3381,6 +3986,11 @@
           <t>대상은?</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
@@ -3398,6 +4008,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
@@ -3415,6 +4030,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
@@ -3432,6 +4052,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
@@ -3449,6 +4074,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
@@ -3471,7 +4101,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E127" s="1" t="inlineStr">
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F127" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3493,6 +4128,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
@@ -3515,7 +4155,12 @@
           <t>소환할 동물은?</t>
         </is>
       </c>
-      <c r="E129" s="1" t="inlineStr">
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F129" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3537,7 +4182,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E130" s="1" t="inlineStr">
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F130" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3564,7 +4214,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E131" s="1" t="inlineStr">
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F131" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3591,7 +4246,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E132" s="1" t="inlineStr">
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F132" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3613,7 +4273,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E133" s="1" t="inlineStr">
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F133" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3640,7 +4305,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E134" s="1" t="inlineStr">
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F134" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3667,7 +4337,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E135" s="1" t="inlineStr">
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F135" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3689,7 +4364,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E136" s="1" t="inlineStr">
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F136" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3716,7 +4396,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E137" s="1" t="inlineStr">
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F137" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3743,7 +4428,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E138" s="1" t="inlineStr">
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F138" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3765,7 +4455,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E139" s="1" t="inlineStr">
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F139" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3792,7 +4487,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E140" s="1" t="inlineStr">
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F140" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3814,6 +4514,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
@@ -3836,7 +4541,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E142" s="1" t="inlineStr">
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F142" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3858,7 +4568,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E143" s="1" t="inlineStr">
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F143" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3880,7 +4595,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E144" s="1" t="inlineStr">
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F144" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3902,7 +4622,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E145" s="1" t="inlineStr">
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F145" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3924,7 +4649,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E146" s="1" t="inlineStr">
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F146" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3946,7 +4676,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E147" s="1" t="inlineStr">
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F147" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -3968,6 +4703,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
@@ -3985,7 +4725,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E149" s="1" t="inlineStr">
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F149" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4012,7 +4757,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E150" s="1" t="inlineStr">
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F150" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4039,7 +4789,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E151" s="1" t="inlineStr">
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F151" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4066,7 +4821,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E152" s="1" t="inlineStr">
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F152" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4088,7 +4848,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E153" s="1" t="inlineStr">
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F153" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4110,7 +4875,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E154" s="1" t="inlineStr">
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F154" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4137,7 +4907,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E155" s="1" t="inlineStr">
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F155" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4164,7 +4939,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E156" s="1" t="inlineStr">
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F156" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4186,7 +4966,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E157" s="1" t="inlineStr">
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F157" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4213,7 +4998,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E158" s="1" t="inlineStr">
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F158" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4240,7 +5030,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E159" s="1" t="inlineStr">
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F159" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4267,7 +5062,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E160" s="1" t="inlineStr">
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F160" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4294,7 +5094,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E161" s="1" t="inlineStr">
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F161" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4321,7 +5126,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E162" s="1" t="inlineStr">
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F162" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4348,7 +5158,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E163" s="1" t="inlineStr">
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F163" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4375,7 +5190,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E164" s="1" t="inlineStr">
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F164" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4402,7 +5222,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E165" s="1" t="inlineStr">
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F165" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4429,7 +5254,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E166" s="1" t="inlineStr">
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F166" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4451,7 +5281,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E167" s="1" t="inlineStr">
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F167" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4473,7 +5308,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E168" s="1" t="inlineStr">
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F168" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4500,7 +5340,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E169" s="1" t="inlineStr">
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F169" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4527,7 +5372,12 @@
           <t>대상은?</t>
         </is>
       </c>
-      <c r="E170" s="1" t="inlineStr">
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F170" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4554,6 +5404,11 @@
           <t>소환할 대상은?</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
@@ -4576,6 +5431,11 @@
           <t>출두할 대상은?</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
@@ -4593,6 +5453,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
@@ -4615,6 +5480,11 @@
           <t>생성할 아이템은?</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
@@ -4637,7 +5507,12 @@
           <t>검색할 맵 이름은?</t>
         </is>
       </c>
-      <c r="E175" s="1" t="inlineStr">
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F175" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4664,7 +5539,12 @@
           <t>할 말은?</t>
         </is>
       </c>
-      <c r="E176" s="1" t="inlineStr">
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F176" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -4691,6 +5571,11 @@
           <t>대상은?</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
@@ -4708,6 +5593,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
@@ -4725,6 +5615,11 @@
           <t>UNKNOWN3</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
@@ -4742,6 +5637,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
@@ -4759,6 +5659,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
@@ -4776,6 +5681,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
@@ -4793,6 +5703,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
@@ -4810,6 +5725,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
@@ -4827,6 +5747,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
@@ -4844,6 +5769,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
@@ -4861,6 +5791,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
@@ -4878,6 +5813,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
@@ -4895,6 +5835,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
@@ -4912,6 +5857,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
@@ -4929,6 +5879,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
@@ -4946,6 +5901,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
@@ -4963,6 +5923,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
@@ -4980,6 +5945,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
@@ -4997,6 +5967,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
@@ -5014,6 +5989,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
@@ -5031,6 +6011,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
@@ -5048,6 +6033,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
@@ -5065,6 +6055,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
@@ -5082,6 +6077,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
@@ -5099,6 +6099,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
@@ -5116,6 +6121,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
@@ -5133,6 +6143,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
@@ -5150,6 +6165,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
@@ -5167,6 +6187,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
@@ -5184,6 +6209,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
@@ -5201,6 +6231,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
@@ -5218,6 +6253,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
@@ -5235,6 +6275,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
@@ -5252,6 +6297,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
@@ -5269,6 +6319,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
@@ -5286,6 +6341,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
@@ -5303,6 +6363,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
@@ -5320,6 +6385,11 @@
           <t>NORMAL</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
@@ -5337,7 +6407,12 @@
           <t>TARGET</t>
         </is>
       </c>
-      <c r="E215" s="1" t="inlineStr">
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F215" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5359,7 +6434,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E216" s="1" t="inlineStr">
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F216" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5381,7 +6461,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E217" s="1" t="inlineStr">
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F217" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5403,7 +6488,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E218" s="1" t="inlineStr">
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F218" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5425,7 +6515,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E219" s="1" t="inlineStr">
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="F219" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5447,7 +6542,12 @@
           <t>TARGET</t>
         </is>
       </c>
-      <c r="E220" s="1" t="inlineStr">
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F220" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5474,7 +6574,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E221" s="1" t="inlineStr">
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F221" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5501,7 +6606,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E222" s="1" t="inlineStr">
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F222" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5528,7 +6638,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E223" s="1" t="inlineStr">
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F223" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5555,7 +6670,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E224" s="1" t="inlineStr">
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F224" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5582,7 +6702,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E225" s="1" t="inlineStr">
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F225" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5609,7 +6734,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E226" s="1" t="inlineStr">
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F226" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5636,7 +6766,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E227" s="1" t="inlineStr">
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F227" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5663,7 +6798,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E228" s="1" t="inlineStr">
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F228" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5690,7 +6830,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E229" s="1" t="inlineStr">
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F229" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5717,7 +6862,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E230" s="1" t="inlineStr">
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F230" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5744,7 +6894,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E231" s="1" t="inlineStr">
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F231" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5771,7 +6926,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E232" s="1" t="inlineStr">
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F232" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5798,7 +6958,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E233" s="1" t="inlineStr">
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F233" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5825,7 +6990,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E234" s="1" t="inlineStr">
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F234" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5852,7 +7022,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E235" s="1" t="inlineStr">
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F235" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5879,7 +7054,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E236" s="1" t="inlineStr">
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F236" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5906,7 +7086,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E237" s="1" t="inlineStr">
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F237" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5933,7 +7118,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E238" s="1" t="inlineStr">
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F238" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5960,7 +7150,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E239" s="1" t="inlineStr">
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F239" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -5987,7 +7182,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E240" s="1" t="inlineStr">
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F240" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6014,7 +7214,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E241" s="1" t="inlineStr">
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F241" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6041,7 +7246,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E242" s="1" t="inlineStr">
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F242" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6068,7 +7278,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E243" s="1" t="inlineStr">
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F243" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6095,7 +7310,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E244" s="1" t="inlineStr">
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F244" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6122,7 +7342,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E245" s="1" t="inlineStr">
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F245" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6149,7 +7374,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E246" s="1" t="inlineStr">
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F246" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6176,7 +7406,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E247" s="1" t="inlineStr">
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F247" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6203,7 +7438,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E248" s="1" t="inlineStr">
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F248" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6230,7 +7470,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E249" s="1" t="inlineStr">
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F249" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6257,7 +7502,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E250" s="1" t="inlineStr">
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F250" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6284,7 +7534,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E251" s="1" t="inlineStr">
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F251" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6311,7 +7566,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E252" s="1" t="inlineStr">
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F252" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6338,7 +7598,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E253" s="1" t="inlineStr">
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F253" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6365,7 +7630,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E254" s="1" t="inlineStr">
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F254" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6392,7 +7662,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E255" s="1" t="inlineStr">
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F255" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6419,7 +7694,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E256" s="1" t="inlineStr">
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F256" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6446,7 +7726,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E257" s="1" t="inlineStr">
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F257" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6473,7 +7758,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E258" s="1" t="inlineStr">
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F258" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6500,7 +7790,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E259" s="1" t="inlineStr">
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F259" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6527,7 +7822,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E260" s="1" t="inlineStr">
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F260" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6549,7 +7849,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E261" s="1" t="inlineStr">
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F261" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6576,7 +7881,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E262" s="1" t="inlineStr">
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F262" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6598,7 +7908,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E263" s="1" t="inlineStr">
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F263" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6620,7 +7935,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E264" s="1" t="inlineStr">
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F264" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6647,7 +7967,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E265" s="1" t="inlineStr">
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F265" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6669,7 +7994,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E266" s="1" t="inlineStr">
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F266" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6691,7 +8021,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E267" s="1" t="inlineStr">
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F267" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6713,7 +8048,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E268" s="1" t="inlineStr">
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F268" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6735,7 +8075,12 @@
           <t>TARGET</t>
         </is>
       </c>
-      <c r="E269" s="1" t="inlineStr">
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F269" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6762,7 +8107,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E270" s="1" t="inlineStr">
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F270" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6789,7 +8139,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E271" s="1" t="inlineStr">
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F271" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6816,7 +8171,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E272" s="1" t="inlineStr">
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F272" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6843,7 +8203,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E273" s="1" t="inlineStr">
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F273" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6870,7 +8235,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E274" s="1" t="inlineStr">
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F274" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6892,7 +8262,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E275" s="1" t="inlineStr">
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F275" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6914,7 +8289,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E276" s="1" t="inlineStr">
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F276" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6936,7 +8316,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E277" s="1" t="inlineStr">
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F277" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6958,7 +8343,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E278" s="1" t="inlineStr">
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F278" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -6980,7 +8370,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E279" s="1" t="inlineStr">
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F279" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7002,7 +8397,12 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="E280" s="1" t="inlineStr">
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F280" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7029,7 +8429,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E281" s="1" t="inlineStr">
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F281" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7056,7 +8461,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E282" s="1" t="inlineStr">
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F282" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7083,7 +8493,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E283" s="1" t="inlineStr">
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F283" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7110,7 +8525,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E284" s="1" t="inlineStr">
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F284" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7137,7 +8557,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E285" s="1" t="inlineStr">
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F285" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7164,7 +8589,12 @@
           <t xml:space="preserve">대상은? </t>
         </is>
       </c>
-      <c r="E286" s="1" t="inlineStr">
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F286" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7191,7 +8621,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E287" s="1" t="inlineStr">
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F287" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7218,7 +8653,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E288" s="1" t="inlineStr">
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F288" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7245,7 +8685,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E289" s="1" t="inlineStr">
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F289" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7272,7 +8717,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E290" s="1" t="inlineStr">
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F290" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7299,7 +8749,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E291" s="1" t="inlineStr">
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F291" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7326,7 +8781,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E292" s="1" t="inlineStr">
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F292" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7353,7 +8813,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E293" s="1" t="inlineStr">
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F293" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7380,7 +8845,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E294" s="1" t="inlineStr">
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F294" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7407,7 +8877,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E295" s="1" t="inlineStr">
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F295" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7434,7 +8909,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E296" s="1" t="inlineStr">
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F296" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7461,7 +8941,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E297" s="1" t="inlineStr">
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F297" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7488,7 +8973,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E298" s="1" t="inlineStr">
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F298" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7515,7 +9005,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E299" s="1" t="inlineStr">
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F299" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -7542,7 +9037,12 @@
           <t xml:space="preserve">변신할 동물은? </t>
         </is>
       </c>
-      <c r="E300" s="1" t="inlineStr">
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>USER</t>
+        </is>
+      </c>
+      <c r="F300" s="1" t="inlineStr">
         <is>
           <t>O</t>
         </is>

</xml_diff>